<commit_message>
auto backup: 2026-03-10 09:50:24
</commit_message>
<xml_diff>
--- a/paper_reading_summary_en.xlsx
+++ b/paper_reading_summary_en.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -604,6 +604,31 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Experimental characterization and thermodynamic mapping of grain boundary segregation in Mg-2Y alloy (metadata-only)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Quantify grain-boundary segregation behavior in Mg-2Y and connect segregation thermodynamics to mechanical behavior and alloy design.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Google Scholar-driven metadata scan; source metadata from Materials Today Communications page. DOI: 10.1016/j.mtla.2025.102584. Access: https://doi.org/10.1016/j.mtla.2025.102584</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Selected as today's candidate due to high topical relevance to Mg alloy, solute segregation, mechanical property, and deformation mechanism. The study experimentally characterizes Y segregation at grain boundaries and maps segregation energetics/thermodynamics. This provides a quantitative basis for linking boundary chemistry to strength-ductility behavior in Mg alloys. No open-access PDF was auto-downloaded in this run, so this entry is metadata-only for manual follow-up reading.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -615,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -657,6 +682,23 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-10 09:45:02 +09:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Daily Paper Scout backfill</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Added 1 metadata-only paper entry to Papers; no downloadable OA PDF found automatically.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>